<commit_message>
use DocLang instance consistently, sync reference.xlsx with spec
Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -543,7 +543,7 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>*Semantic elements* capture core components with specific meaning and functional role in the document (e.g. a paragraph, a table, a list etc.) and may optionally begin with a [element head](#element-head).
+          <t>*Semantic elements* capture core document components with specific meaning and functional role (e.g. a paragraph, a table, a list etc.) and may optionally begin with a [element head](#element-head).
 They are generally meant to be interpreted as block-level elements (although they can also be inlined via nesting).
 Semantic elements that can appear on the top level within `&lt;doclang&gt;` are called *primary*, while those that can only appear within other semantic elements are called *secondary*.</t>
         </is>
@@ -766,7 +766,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Indicates a page break. A paginated document may be divided into pages using the `&lt;page_break/&gt;` empty element. Any page content, as split by `&lt;page_break/&gt;`, forms a valid DocLang [document body](#head-and-body-areas), i.e. would be a valid DocLang document if wrapped in a `doclang` root element.</t>
+          <t>Indicates a page break. A paginated document may be divided into pages using the `&lt;page_break/&gt;` empty element. Any page content, as split by `&lt;page_break/&gt;`, forms a valid DocLang [document body](#head-and-body-areas), i.e. would be a valid DocLang instance if wrapped in a `doclang` root element.</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
@@ -1516,7 +1516,7 @@
       <c r="C24" s="5" t="inlineStr">
         <is>
           <t>Optional part of the element head for capturing an associated caption. Unlike `&lt;description&gt;` or `&lt;summary&gt;`, `&lt;caption&gt;` is an actual
-document component, which can have its own location information etc. For example, a caption shown underneath a chart.</t>
+document component, which can have its own location information etc. For example, a caption shown underneath a chart. An element head may contain multiple captions, e.g. a figure with both a title above and a note below, or the same caption in several languages.</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -1932,7 +1932,7 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>The conceptual layer of the host element in the document.</t>
+          <t>The conceptual layer of the host element in the DocLang instance.</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
@@ -2965,7 +2965,7 @@
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>Defines the default resolution for the document.</t>
+          <t>Defines the default resolution for the DocLang instance.</t>
         </is>
       </c>
       <c r="D64" s="6" t="inlineStr">
@@ -4067,7 +4067,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>The DocLang specification version the document is supposed to validate against, in "MAJOR.MINOR" format, i.e. first two positions of Semantic Verisoning.</t>
+          <t>The DocLang specification version the DocLang instance is supposed to validate against, in "MAJOR.MINOR" format, i.e. first two positions of Semantic Verisoning.</t>
         </is>
       </c>
     </row>
@@ -4202,7 +4202,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>The layer value: "body" is for the document's main content, "background" is for watermarks and other background components, while "furniture" is the fallback for any supplementary components not contributing to the document's main content, such as navigation or decorations.</t>
+          <t>The layer value: "body" is for the main content, "background" is for watermarks and other background components, while "furniture" is the fallback for any supplementary components not contributing to the main content, such as navigation or decorations.</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>The ID of the referenced thread. This must be defined by at least one `&lt;thread&gt;` in the document.</t>
+          <t>The ID of the referenced thread. This must be defined by at least one `&lt;thread&gt;` in the DocLang instance.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
specify version as unspecified when omitted
Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -4057,17 +4057,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Optional; default: "0.7"</t>
+          <t>Optional; if omitted, the version is unspecified</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>{"0.7"}</t>
+          <t>"MAJOR.MINOR" of a published DocLang specification version</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>The DocLang specification version the DocLang instance is supposed to validate against, in "MAJOR.MINOR" format, i.e. first two positions of Semantic Verisoning.</t>
+          <t>The DocLang specification version the DocLang instance is supposed to validate against, in "MAJOR.MINOR" format, i.e. first two positions of Semantic Versioning. If omitted, the version is unspecified (see [Omitted version](#omitted-version)).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
use single-line annex headings and update links to them
Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -1182,7 +1182,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Captures a code snippet, either as a standalone block or inlined within a semantic element. For language classification, use a `&lt;label&gt;`in the element head (see [Recommendations](#recommendations)).</t>
+          <t>Captures a code snippet, either as a standalone block or inlined within a semantic element. For language classification, use a `&lt;label&gt;`in the element head (see [Recommendations](#annex-c-informative-recommendations)).</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Optional part of the element head; custom metadata, e.g. for application-specific purposes. See [Recommendations](#recommendations) for naming and namespacing guidance for custom vocabularies.</t>
+          <t>Optional part of the element head; custom metadata, e.g. for application-specific purposes. See [Recommendations](#annex-c-informative-recommendations) for naming and namespacing guidance for custom vocabularies.</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">

</xml_diff>

<commit_message>
allow semantic elements in transcript turns
Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -800,7 +800,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Represents a piece of cohesive text as that would appear in a paragraph. Note: a special construct related to this element is the so-called "virtual `&lt;text&gt;`", which can occur only as a list item or a table cell — see `&lt;list&gt;` and `&lt;table&gt;` below for details.</t>
+          <t>Represents a piece of cohesive text as that would appear in a paragraph. Note: a special construct related to this element is the so-called "virtual `&lt;text&gt;`", which can occur only as a list item, a table cell or a transcript turn — see [Lists](#lists).</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -1022,7 +1022,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Captures a list. List items are started by the respective structural elements (`&lt;ldiv&gt;`). A non-empty `&lt;list&gt;` element body must begin with such a structural element. A list item can be defined without a wrapping tag, i.e. as pure (optional) element head followed by raw text; this is called an "virtual `&lt;text&gt;`" and is handled exactly like a regular `&lt;text&gt;` element.</t>
+          <t>Captures a list. List items are started by the respective structural elements (`&lt;ldiv&gt;`). A non-empty `&lt;list&gt;` element body must begin with such a structural element. Each list item can be any semantic element sequence or a virtual `&lt;text&gt;`.</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -1063,7 +1063,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Captures a table in an OTSL-based format. Table cells are started by the respective structural elements (`&lt;fcel&gt;` etc). A non-empty `&lt;table&gt;` element body must begin with such a structural element. A table cell can be defined without a wrapping tag, i.e. as pure (optional) element head followed by raw text; this is called an "virtual `&lt;text&gt;`" and is handled exactly like a regular `&lt;text&gt;` element.</t>
+          <t>Captures a table in an OTSL-based format. Table cells are started by the respective structural elements (`&lt;fcel&gt;` etc). A non-empty `&lt;table&gt;` element body must begin with such a structural element. Each table cell can be any semantic element sequence or a virtual `&lt;text&gt;`.</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Captures an index, e.g. for a table of contents or glossary, in an OTSL-based format. Index cells are started by the respective structural elements (`&lt;fcel&gt;` etc). A non-empty `&lt;index&gt;` element body must begin with such a structural element. A cell can be defined without a wrapping tag, i.e. as pure (optional) element head followed by raw text; this is called an "virtual `&lt;text&gt;`" and is handled exactly like a regular `&lt;text&gt;` element.</t>
+          <t>Captures an index, e.g. for a table of contents or glossary, in an OTSL-based format. Index cells are started by the respective structural elements (`&lt;fcel&gt;` etc). A non-empty `&lt;index&gt;` element body must begin with such a structural element. Each cell can be any semantic element sequence or a virtual `&lt;text&gt;`.</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -3584,7 +3584,7 @@
       </c>
       <c r="C78" s="1" t="inlineStr">
         <is>
-          <t>Captures a time-aligned media transcript (subtitles, captions, or diarized speech). The body may open with a single `&lt;cover&gt;` (a track-wide image), then a sequence of cue blocks, each introduced by a `&lt;bdiv&gt;` delimiter; a non-empty `&lt;track&gt;` body must begin with a `&lt;cover&gt;` or a `&lt;bdiv&gt;`. A cue block carries a mandatory start time, an optional end time (each a run of `&lt;hours&gt;`/`&lt;minutes&gt;`/`&lt;seconds&gt;`/`&lt;msecs&gt;`), an optional `&lt;chapter&gt;`, an optional `&lt;frame&gt;`, an optional `&lt;audio&gt;`, and an optional transcript of `&lt;voice&gt;`-attributed turns.</t>
+          <t>Captures a time-aligned media transcript (subtitles, captions, or diarized speech). The body may open with a single `&lt;cover&gt;` (a track-wide image), then a sequence of cue blocks, each introduced by a `&lt;bdiv&gt;` delimiter; a non-empty `&lt;track&gt;` body must begin with a `&lt;cover&gt;` or a `&lt;bdiv&gt;`. A cue block carries a mandatory start time, an optional end time (each a run of `&lt;hours&gt;`/`&lt;minutes&gt;`/`&lt;seconds&gt;`/`&lt;msecs&gt;`), an optional `&lt;chapter&gt;`, an optional `&lt;frame&gt;`, an optional `&lt;audio&gt;`, and an optional transcript of turns, each an optional `&lt;voice&gt;` followed by its content, which can be any semantic element sequence or a virtual `&lt;text&gt;`.</t>
         </is>
       </c>
       <c r="D78" s="1" t="inlineStr">
@@ -3595,17 +3595,19 @@
       <c r="E78" t="b">
         <v>1</v>
       </c>
-      <c r="F78" s="1" t="b">
-        <v>1</v>
+      <c r="F78" s="1" t="inlineStr">
+        <is>
+          <t>TRUE, also on transcript turn level in case of virtual `&lt;text&gt;`</t>
+        </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Only within a cue block transcript</t>
+          <t>Only on transcript turn level, in case of virtual `&lt;text&gt;`</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>`&lt;cover&gt;` before the first cue block; within cue blocks, `&lt;chapter&gt;`, `&lt;frame&gt;`, `&lt;audio&gt;`, and `&lt;voice&gt;`</t>
+          <t>`&lt;cover&gt;` before the first cue block; within cue blocks, `&lt;chapter&gt;`, `&lt;frame&gt;`, `&lt;audio&gt;` and `&lt;voice&gt;`; on transcript turn level, any</t>
         </is>
       </c>
       <c r="I78" t="b">

</xml_diff>

<commit_message>
define whitespace handling (#205)
* define whitespace handling

Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>

* add whitespace migration step

Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>

* add whitespace downgrade step

Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>

---------

Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -544,7 +544,7 @@
       <c r="B3" s="8" t="inlineStr">
         <is>
           <t>*Semantic elements* capture core document components with specific meaning and functional role (e.g. a paragraph, a table, a list etc.) and may optionally begin with a [element head](#element-head).
-They are generally meant to be interpreted as block-level elements (although they can also be inlined via nesting).
+They are generally meant to be read as separate blocks, such as a paragraph, although some can also be nested within text.
 Semantic elements that can appear on the top level within `&lt;doclang&gt;` are called *primary*, while those that can only appear within other semantic elements are called *secondary*.</t>
         </is>
       </c>
@@ -800,7 +800,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Represents a piece of cohesive text as that would appear in a paragraph. Note: a special construct related to this element is the so-called "virtual `&lt;text&gt;`", which can occur only as a list item or a table cell — see `&lt;list&gt;` and `&lt;table&gt;` below for details.</t>
+          <t>Represents a piece of cohesive text as that would appear in a paragraph. A list item, or a cell of a `&lt;table&gt;`, `&lt;index&gt;` or `&lt;tabular&gt;`, may also consist of raw text, optionally preceded by an element head, without wrapping `&lt;text&gt;` tags. Such content is called a *virtual `&lt;text&gt;`* and is interpreted exactly as if it were wrapped in `&lt;text&gt;` tags.</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -1022,7 +1022,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Captures a list. List items are started by the respective structural elements (`&lt;ldiv&gt;`). A non-empty `&lt;list&gt;` element body must begin with such a structural element. A list item can be defined without a wrapping tag, i.e. as pure (optional) element head followed by raw text; this is called an "virtual `&lt;text&gt;`" and is handled exactly like a regular `&lt;text&gt;` element.</t>
+          <t>Captures a list. List items are started by the respective structural elements (`&lt;ldiv&gt;`). A non-empty `&lt;list&gt;` element body must begin with such a structural element. A list item can be any semantic element sequence or a virtual `&lt;text&gt;`.</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -1063,7 +1063,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Captures a table in an OTSL-based format. Table cells are started by the respective structural elements (`&lt;fcel&gt;` etc). A non-empty `&lt;table&gt;` element body must begin with such a structural element. A table cell can be defined without a wrapping tag, i.e. as pure (optional) element head followed by raw text; this is called an "virtual `&lt;text&gt;`" and is handled exactly like a regular `&lt;text&gt;` element.</t>
+          <t>Captures a table in an OTSL-based format. Table cells are started by the respective structural elements (`&lt;fcel&gt;` etc). A non-empty `&lt;table&gt;` element body must begin with such a structural element. A table cell can be any semantic element sequence or a virtual `&lt;text&gt;`.</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Captures an index, e.g. for a table of contents or glossary, in an OTSL-based format. Index cells are started by the respective structural elements (`&lt;fcel&gt;` etc). A non-empty `&lt;index&gt;` element body must begin with such a structural element. A cell can be defined without a wrapping tag, i.e. as pure (optional) element head followed by raw text; this is called an "virtual `&lt;text&gt;`" and is handled exactly like a regular `&lt;text&gt;` element.</t>
+          <t>Captures an index, e.g. for a table of contents or glossary, in an OTSL-based format. Index cells are started by the respective structural elements (`&lt;fcel&gt;` etc). A non-empty `&lt;index&gt;` element body must begin with such a structural element. A cell can be any semantic element sequence or a virtual `&lt;text&gt;`.</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">

</xml_diff>